<commit_message>
Added server API attributes
</commit_message>
<xml_diff>
--- a/data/Influencers Sheet.xlsx
+++ b/data/Influencers Sheet.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t xml:space="preserve">USERNAME </t>
   </si>
@@ -34,58 +34,16 @@
     <t xml:space="preserve">Name </t>
   </si>
   <si>
-    <t xml:space="preserve">anshi_lifestyle316</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.instagram.com/anshi_lifestyle316?utm_source=ig_web_button_share_sheet&amp;igsh=ZDNlZDc0MzIxNw==</t>
-  </si>
-  <si>
-    <t xml:space="preserve">agarwalanshi33@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mridul tripathi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.instagram.com/mridultripathi_</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mridultripathi23@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">anjali_s08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.instagram.com/anjali_s08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cinnamonblush08@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">akankshasoni1897</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.instagram.com/akankshasoni1897?utm_source=ig_web_button_share_sheet&amp;igsh=ZDNlZDc0MzIxNw==</t>
-  </si>
-  <si>
-    <t xml:space="preserve">akankshasoni253@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dishasingh__24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.instagram.com/dishasingh__24/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dishasingh024@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">passion_for_beauty9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.instagram.com/passion_for_beauty9/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prettyfind01@gmail.com</t>
+    <t xml:space="preserve">coder_akram.khan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.instagram.com/coder_akram.khan/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">akram.codes.it@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Akram</t>
   </si>
 </sst>
 </file>
@@ -326,9 +284,9 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:X7"/>
-  <sheetFormatPr defaultColWidth="12.640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.66015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="108.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1023" style="0" width="11.52"/>
@@ -368,7 +326,7 @@
       <c r="W1" s="2"/>
       <c r="X1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -378,7 +336,9 @@
       <c r="C2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="2"/>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -400,16 +360,10 @@
       <c r="W2" s="2"/>
       <c r="X2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>9</v>
-      </c>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="5"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
@@ -432,16 +386,10 @@
       <c r="W3" s="2"/>
       <c r="X3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>12</v>
-      </c>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
@@ -464,16 +412,10 @@
       <c r="W4" s="2"/>
       <c r="X4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>15</v>
-      </c>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="8"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -496,16 +438,10 @@
       <c r="W5" s="2"/>
       <c r="X5" s="2"/>
     </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>18</v>
-      </c>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="5"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -528,16 +464,10 @@
       <c r="W6" s="2"/>
       <c r="X6" s="2"/>
     </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>21</v>
-      </c>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="5"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -562,12 +492,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="https://www.instagram.com/anshi_lifestyle316?utm_source=ig_web_button_share_sheet&amp;igsh=ZDNlZDc0MzIxNw=="/>
-    <hyperlink ref="B3" r:id="rId2" display="https://www.instagram.com/mridultripathi_"/>
-    <hyperlink ref="B4" r:id="rId3" display="https://www.instagram.com/anjali_s08"/>
-    <hyperlink ref="B5" r:id="rId4" display="https://www.instagram.com/akankshasoni1897?utm_source=ig_web_button_share_sheet&amp;igsh=ZDNlZDc0MzIxNw=="/>
-    <hyperlink ref="B6" r:id="rId5" display="https://www.instagram.com/dishasingh__24/"/>
-    <hyperlink ref="B7" r:id="rId6" display="https://www.instagram.com/passion_for_beauty9/"/>
+    <hyperlink ref="C2" r:id="rId1" display="akram.codes.it@gmail.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>